<commit_message>
20-mm data pull code error fix
</commit_message>
<xml_diff>
--- a/data_raw/smelt/2026 20-mm DS and LFS Reporting3.30.26.xlsx
+++ b/data_raw/smelt/2026 20-mm DS and LFS Reporting3.30.26.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://doimspp-my.sharepoint.com/personal/lmccormick_usbr_gov/Documents/Documents/Research/R/samt_smt_assessments/data_raw/smelt/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:1_{2620A007-24F9-4CFE-AB21-1C70F7A2557D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B1462896-62F5-49EC-8E90-DF845C684A03}"/>
+  <xr:revisionPtr revIDLastSave="3" documentId="13_ncr:1_{2620A007-24F9-4CFE-AB21-1C70F7A2557D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D103ECFF-DC37-4DE6-9DE6-DDC0C803906A}"/>
   <bookViews>
-    <workbookView xWindow="2688" yWindow="624" windowWidth="18504" windowHeight="12336" tabRatio="844" xr2:uid="{FADF9BD8-084D-4A05-925F-CF581A2A38ED}"/>
+    <workbookView xWindow="2304" yWindow="624" windowWidth="18504" windowHeight="12336" tabRatio="844" xr2:uid="{FADF9BD8-084D-4A05-925F-CF581A2A38ED}"/>
   </bookViews>
   <sheets>
     <sheet name="Survey 1" sheetId="52" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="29">
   <si>
     <t>Year</t>
   </si>
@@ -178,45 +178,6 @@
   <si>
     <t>Processing is complete through 3/30/26</t>
   </si>
-  <si>
-    <r>
-      <t>901</t>
-    </r>
-    <r>
-      <rPr>
-        <vertAlign val="superscript"/>
-        <sz val="14"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>∆≠</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>902</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>*</t>
-    </r>
-    <r>
-      <rPr>
-        <vertAlign val="superscript"/>
-        <sz val="14"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>∆</t>
-    </r>
-  </si>
 </sst>
 </file>
 
@@ -224,8 +185,8 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="3">
     <numFmt numFmtId="164" formatCode="dd\-mmm\-yy"/>
-    <numFmt numFmtId="166" formatCode="0.0"/>
-    <numFmt numFmtId="167" formatCode="m/d/yy;@"/>
+    <numFmt numFmtId="165" formatCode="0.0"/>
+    <numFmt numFmtId="166" formatCode="m/d/yy;@"/>
   </numFmts>
   <fonts count="9" x14ac:knownFonts="1">
     <font>
@@ -1105,14 +1066,14 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="6" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="167" fontId="6" fillId="21" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="6" fillId="21" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="1" fontId="6" fillId="21" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1133,10 +1094,10 @@
     <xf numFmtId="0" fontId="6" fillId="22" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="166" fontId="6" fillId="22" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="6" fillId="21" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="6" fillId="22" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="6" fillId="21" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="1" fontId="6" fillId="21" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1157,10 +1118,10 @@
     <xf numFmtId="0" fontId="6" fillId="22" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="166" fontId="6" fillId="22" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="6" fillId="16" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="6" fillId="22" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="6" fillId="16" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="1" fontId="6" fillId="16" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1181,13 +1142,13 @@
     <xf numFmtId="0" fontId="6" fillId="9" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="166" fontId="6" fillId="9" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="6" fillId="16" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="167" fontId="6" fillId="16" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="6" fillId="9" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="6" fillId="16" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="6" fillId="16" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="1" fontId="6" fillId="16" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1205,7 +1166,7 @@
     <xf numFmtId="0" fontId="6" fillId="9" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="166" fontId="6" fillId="9" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="6" fillId="9" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="9" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1220,7 +1181,7 @@
     <xf numFmtId="0" fontId="6" fillId="12" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="167" fontId="6" fillId="12" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="6" fillId="12" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="1" fontId="6" fillId="12" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1241,7 +1202,7 @@
     <xf numFmtId="0" fontId="6" fillId="20" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="167" fontId="6" fillId="12" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="6" fillId="12" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="1" fontId="6" fillId="12" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1262,7 +1223,7 @@
     <xf numFmtId="0" fontId="6" fillId="12" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="167" fontId="6" fillId="12" borderId="40" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="6" fillId="12" borderId="40" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="1" fontId="6" fillId="12" borderId="40" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1283,7 +1244,7 @@
     <xf numFmtId="0" fontId="6" fillId="19" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="167" fontId="6" fillId="19" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="6" fillId="19" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="1" fontId="6" fillId="19" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1298,7 +1259,7 @@
     <xf numFmtId="0" fontId="6" fillId="13" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="166" fontId="6" fillId="13" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="6" fillId="13" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="19" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1307,7 +1268,7 @@
     <xf numFmtId="0" fontId="6" fillId="13" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="167" fontId="6" fillId="19" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="6" fillId="19" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="1" fontId="6" fillId="19" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1322,7 +1283,7 @@
     <xf numFmtId="0" fontId="6" fillId="13" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="166" fontId="6" fillId="13" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="6" fillId="13" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="19" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1334,7 +1295,7 @@
     <xf numFmtId="0" fontId="6" fillId="13" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="167" fontId="6" fillId="19" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="6" fillId="19" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="1" fontId="6" fillId="19" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1349,7 +1310,7 @@
     <xf numFmtId="0" fontId="6" fillId="13" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="166" fontId="6" fillId="13" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="6" fillId="13" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="15" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1358,7 +1319,7 @@
     <xf numFmtId="0" fontId="6" fillId="18" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="167" fontId="6" fillId="18" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="6" fillId="18" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="1" fontId="6" fillId="18" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1373,7 +1334,7 @@
     <xf numFmtId="0" fontId="6" fillId="15" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="166" fontId="6" fillId="15" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="6" fillId="15" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="18" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1382,7 +1343,7 @@
     <xf numFmtId="0" fontId="6" fillId="15" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="167" fontId="6" fillId="18" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="6" fillId="18" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="1" fontId="6" fillId="15" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1394,7 +1355,7 @@
     <xf numFmtId="0" fontId="6" fillId="15" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="166" fontId="6" fillId="15" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="6" fillId="15" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="18" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1403,7 +1364,7 @@
     <xf numFmtId="0" fontId="6" fillId="15" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="167" fontId="6" fillId="15" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="6" fillId="15" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="1" fontId="6" fillId="15" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1418,7 +1379,7 @@
     <xf numFmtId="0" fontId="6" fillId="15" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="166" fontId="6" fillId="15" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="6" fillId="15" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="17" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1427,7 +1388,7 @@
     <xf numFmtId="0" fontId="6" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="167" fontId="6" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="6" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="1" fontId="6" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1442,7 +1403,7 @@
     <xf numFmtId="0" fontId="6" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="166" fontId="6" fillId="2" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="6" fillId="2" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="17" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1451,7 +1412,7 @@
     <xf numFmtId="0" fontId="6" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="167" fontId="6" fillId="2" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="6" fillId="2" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="1" fontId="6" fillId="2" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1466,10 +1427,10 @@
     <xf numFmtId="0" fontId="6" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="166" fontId="6" fillId="2" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="6" fillId="8" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="6" fillId="2" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="6" fillId="8" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="1" fontId="6" fillId="8" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1484,7 +1445,7 @@
     <xf numFmtId="0" fontId="6" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="167" fontId="6" fillId="8" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="6" fillId="8" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="1" fontId="6" fillId="8" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1502,7 +1463,7 @@
     <xf numFmtId="0" fontId="6" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="166" fontId="6" fillId="2" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="6" fillId="2" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1511,7 +1472,7 @@
     <xf numFmtId="0" fontId="6" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="167" fontId="6" fillId="7" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="6" fillId="7" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="1" fontId="6" fillId="7" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1529,13 +1490,13 @@
     <xf numFmtId="0" fontId="6" fillId="3" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="166" fontId="6" fillId="3" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="6" fillId="3" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="167" fontId="6" fillId="7" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="6" fillId="7" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="1" fontId="6" fillId="7" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1553,7 +1514,7 @@
     <xf numFmtId="0" fontId="6" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="166" fontId="6" fillId="3" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="6" fillId="3" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1562,7 +1523,7 @@
     <xf numFmtId="0" fontId="6" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="167" fontId="6" fillId="7" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="6" fillId="7" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="1" fontId="6" fillId="7" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1580,7 +1541,7 @@
     <xf numFmtId="0" fontId="6" fillId="3" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="166" fontId="6" fillId="3" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="6" fillId="3" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="6" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1589,7 +1550,7 @@
     <xf numFmtId="0" fontId="6" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="167" fontId="6" fillId="6" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="6" fillId="6" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="1" fontId="6" fillId="6" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1610,7 +1571,7 @@
     <xf numFmtId="0" fontId="6" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="166" fontId="6" fillId="4" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="6" fillId="4" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1619,7 +1580,7 @@
     <xf numFmtId="0" fontId="6" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="167" fontId="6" fillId="6" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="6" fillId="6" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="1" fontId="6" fillId="6" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1634,7 +1595,7 @@
     <xf numFmtId="0" fontId="6" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="166" fontId="6" fillId="4" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="6" fillId="4" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="14" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1643,7 +1604,7 @@
     <xf numFmtId="0" fontId="6" fillId="11" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="167" fontId="6" fillId="14" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="6" fillId="14" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="1" fontId="6" fillId="14" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1661,7 +1622,7 @@
     <xf numFmtId="0" fontId="6" fillId="11" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="166" fontId="6" fillId="11" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="6" fillId="11" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="6" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1670,13 +1631,13 @@
     <xf numFmtId="0" fontId="6" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="6" fillId="6" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="6" fillId="6" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="167" fontId="6" fillId="6" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="6" fillId="6" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="1" fontId="6" fillId="6" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1694,7 +1655,7 @@
     <xf numFmtId="0" fontId="6" fillId="4" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="166" fontId="6" fillId="4" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="6" fillId="4" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1719,31 +1680,31 @@
     <xf numFmtId="0" fontId="5" fillId="5" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="5" fillId="5" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="5" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="6" fillId="12" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="6" fillId="12" borderId="44" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="6" fillId="10" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="6" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="6" fillId="12" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="12" borderId="44" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="10" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="167" fontId="7" fillId="12" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="7" fillId="12" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="1" fontId="7" fillId="12" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1761,10 +1722,10 @@
     <xf numFmtId="0" fontId="7" fillId="12" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="166" fontId="7" fillId="12" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="7" fillId="12" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="7" fillId="12" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="12" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="16" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1809,7 +1770,7 @@
     <xf numFmtId="0" fontId="6" fillId="26" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="167" fontId="6" fillId="25" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="6" fillId="25" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="1" fontId="6" fillId="25" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1827,91 +1788,91 @@
     <xf numFmtId="0" fontId="6" fillId="26" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="166" fontId="6" fillId="26" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="5" fillId="5" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="6" fillId="26" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="5" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="6" fillId="12" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="7" fillId="12" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="6" fillId="12" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="6" fillId="12" borderId="40" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="6" fillId="19" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="6" fillId="19" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="6" fillId="19" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="6" fillId="18" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="6" fillId="15" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="6" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="6" fillId="2" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="6" fillId="8" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="6" fillId="8" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="6" fillId="7" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="6" fillId="7" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="6" fillId="7" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="6" fillId="6" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="6" fillId="6" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="6" fillId="14" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="6" fillId="6" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="6" fillId="21" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="6" fillId="21" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="6" fillId="16" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="6" fillId="16" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="6" fillId="25" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="6" fillId="16" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="6" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="6" fillId="12" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="12" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="12" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="12" borderId="40" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="19" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="19" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="19" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="18" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="15" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="2" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="8" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="8" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="7" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="7" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="7" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="6" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="6" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="14" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="6" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="21" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="21" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="16" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="16" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="25" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="16" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
@@ -2020,6 +1981,10 @@
     <xdr:clientData/>
   </xdr:oneCellAnchor>
 </xdr:wsDr>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3899,8 +3864,8 @@
         <f>C3</f>
         <v>1</v>
       </c>
-      <c r="D55" s="50" t="s">
-        <v>29</v>
+      <c r="D55" s="50">
+        <v>901</v>
       </c>
       <c r="E55" s="42">
         <v>46098</v>
@@ -3937,8 +3902,8 @@
         <f>C3</f>
         <v>1</v>
       </c>
-      <c r="D56" s="50" t="s">
-        <v>30</v>
+      <c r="D56" s="50">
+        <v>902</v>
       </c>
       <c r="E56" s="42">
         <v>46098</v>

</xml_diff>